<commit_message>
New replicate for PN23
</commit_message>
<xml_diff>
--- a/data/PN23/rep2/summary flowcyto with events.xlsx
+++ b/data/PN23/rep2/summary flowcyto with events.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/storage/hien/Hien PhD project new/Result/Full lab evolution exp/mcr1 plasmid/2nd rep/20260330/Flowcytometry/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/storage/hien/Hien PhD project new/Result/Full lab evolution exp/mcr1 plasmid/3rd rep/20260527/Flow cytometry/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AF0E2F3-EF50-E740-92A8-9739CF5A4C1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5186225A-4310-3849-9D2E-8306E0E244EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="19460" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="19460" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="114">
   <si>
     <t>vial</t>
   </si>
@@ -57,205 +57,316 @@
     <t>M5</t>
   </si>
   <si>
-    <t>M6</t>
-  </si>
-  <si>
-    <t>M7</t>
-  </si>
-  <si>
-    <t>28,1 %</t>
-  </si>
-  <si>
     <t>Events</t>
   </si>
   <si>
-    <t>13,5 %</t>
-  </si>
-  <si>
     <t>22,1 %</t>
   </si>
   <si>
-    <t>31,2 %</t>
-  </si>
-  <si>
-    <t>37,9 %</t>
-  </si>
-  <si>
-    <t>26,0 %</t>
-  </si>
-  <si>
-    <t>22h</t>
-  </si>
-  <si>
-    <t>166h</t>
-  </si>
-  <si>
     <t>0h</t>
   </si>
   <si>
-    <t>34,8 %</t>
-  </si>
-  <si>
-    <t>33,4 %</t>
-  </si>
-  <si>
-    <t>24,7 %</t>
-  </si>
-  <si>
-    <t>46,5 %</t>
-  </si>
-  <si>
-    <t>40,3 %</t>
-  </si>
-  <si>
     <t>16,8 %</t>
   </si>
   <si>
-    <t>25,0 %</t>
-  </si>
-  <si>
-    <t>36,5 %</t>
-  </si>
-  <si>
-    <t>34,3 %</t>
-  </si>
-  <si>
-    <t>39,7 %</t>
-  </si>
-  <si>
-    <t>31,6 %</t>
-  </si>
-  <si>
-    <t>24,5 %</t>
-  </si>
-  <si>
-    <t>49,2 %</t>
-  </si>
-  <si>
-    <t>20,2 %</t>
-  </si>
-  <si>
-    <t>15,6 %</t>
-  </si>
-  <si>
-    <t>25,1 %</t>
-  </si>
-  <si>
-    <t>49,9 %</t>
-  </si>
-  <si>
-    <t>14,3 %</t>
-  </si>
-  <si>
-    <t>9,56 %</t>
-  </si>
-  <si>
-    <t>68,7 %</t>
-  </si>
-  <si>
-    <t>7,70 %</t>
-  </si>
-  <si>
-    <t>2,42 %</t>
-  </si>
-  <si>
-    <t>72,0 %</t>
-  </si>
-  <si>
-    <t>94h</t>
-  </si>
-  <si>
-    <t>33,8 %</t>
-  </si>
-  <si>
-    <t>59,6 %</t>
-  </si>
-  <si>
-    <t>4,32 %</t>
-  </si>
-  <si>
-    <t>35,5 %</t>
-  </si>
-  <si>
-    <t>48,4 %</t>
-  </si>
-  <si>
-    <t>11,9 %</t>
-  </si>
-  <si>
-    <t>36,9 %</t>
-  </si>
-  <si>
     <t>53,5 %</t>
   </si>
   <si>
-    <t>6,64 %</t>
-  </si>
-  <si>
-    <t>28,5 %</t>
-  </si>
-  <si>
-    <t>63,2 %</t>
-  </si>
-  <si>
-    <t>3,38 %</t>
-  </si>
-  <si>
-    <t>52,4 %</t>
-  </si>
-  <si>
-    <t>27,8 %</t>
-  </si>
-  <si>
-    <t>12,5 %</t>
-  </si>
-  <si>
-    <t>22,9 %</t>
-  </si>
-  <si>
-    <t>57,7 %</t>
-  </si>
-  <si>
-    <t>12,4 %</t>
-  </si>
-  <si>
-    <t>2,83 %</t>
-  </si>
-  <si>
     <t>70,7 %</t>
   </si>
   <si>
-    <t>47,7 %</t>
-  </si>
-  <si>
-    <t>8,20 %</t>
-  </si>
-  <si>
-    <t>38,4 %</t>
-  </si>
-  <si>
-    <t>43,4 %</t>
-  </si>
-  <si>
-    <t>7,26 %</t>
-  </si>
-  <si>
-    <t>65,4 %</t>
-  </si>
-  <si>
-    <t>20,8 %</t>
-  </si>
-  <si>
-    <t>6,10 %</t>
-  </si>
-  <si>
-    <t>28,0 %</t>
-  </si>
-  <si>
-    <t>63,1 %</t>
-  </si>
-  <si>
-    <t>4,35 %</t>
+    <t>M0</t>
+  </si>
+  <si>
+    <t>18,1 %</t>
+  </si>
+  <si>
+    <t>15,7 %</t>
+  </si>
+  <si>
+    <t>65,7 %</t>
+  </si>
+  <si>
+    <t>23,8 %</t>
+  </si>
+  <si>
+    <t>20,9 %</t>
+  </si>
+  <si>
+    <t>54,7 %</t>
+  </si>
+  <si>
+    <t>18,6 %</t>
+  </si>
+  <si>
+    <t>59,9 %</t>
+  </si>
+  <si>
+    <t>19,9 %</t>
+  </si>
+  <si>
+    <t>19,3 %</t>
+  </si>
+  <si>
+    <t>60,1 %</t>
+  </si>
+  <si>
+    <t>24,6 %</t>
+  </si>
+  <si>
+    <t>52,6 %</t>
+  </si>
+  <si>
+    <t>13,7 %</t>
+  </si>
+  <si>
+    <t>14,2 %</t>
+  </si>
+  <si>
+    <t>68h</t>
+  </si>
+  <si>
+    <t>39,5 %</t>
+  </si>
+  <si>
+    <t>50,7 %</t>
+  </si>
+  <si>
+    <t>7,53 %</t>
+  </si>
+  <si>
+    <t>40,0 %</t>
+  </si>
+  <si>
+    <t>49,4 %</t>
+  </si>
+  <si>
+    <t>8,79 %</t>
+  </si>
+  <si>
+    <t>37,2 %</t>
+  </si>
+  <si>
+    <t>23,4 %</t>
+  </si>
+  <si>
+    <t>36,1 %</t>
+  </si>
+  <si>
+    <t>11,2 %</t>
+  </si>
+  <si>
+    <t>7,25 %</t>
+  </si>
+  <si>
+    <t>78,3 %</t>
+  </si>
+  <si>
+    <t>21,2 %</t>
+  </si>
+  <si>
+    <t>12,2 %</t>
+  </si>
+  <si>
+    <t>54,6 %</t>
+  </si>
+  <si>
+    <t>0,18 %</t>
+  </si>
+  <si>
+    <t>0,041 %</t>
+  </si>
+  <si>
+    <t>90,4 %</t>
+  </si>
+  <si>
+    <t>45,0 %</t>
+  </si>
+  <si>
+    <t>3,36 %</t>
+  </si>
+  <si>
+    <t>55,8 %</t>
+  </si>
+  <si>
+    <t>32,8 %</t>
+  </si>
+  <si>
+    <t>9,30 %</t>
+  </si>
+  <si>
+    <t>39,4 %</t>
+  </si>
+  <si>
+    <t>1,74 %</t>
+  </si>
+  <si>
+    <t>53,3 %</t>
+  </si>
+  <si>
+    <t>37,7 %</t>
+  </si>
+  <si>
+    <t>6,65 %</t>
+  </si>
+  <si>
+    <t>18,4 %</t>
+  </si>
+  <si>
+    <t>11,1 %</t>
+  </si>
+  <si>
+    <t>59,1 %</t>
+  </si>
+  <si>
+    <t>0,090 %</t>
+  </si>
+  <si>
+    <t>0,030 %</t>
+  </si>
+  <si>
+    <t>90,1 %</t>
+  </si>
+  <si>
+    <t>140h</t>
+  </si>
+  <si>
+    <t>44,3 %</t>
+  </si>
+  <si>
+    <t>52,9 %</t>
+  </si>
+  <si>
+    <t>0,90 %</t>
+  </si>
+  <si>
+    <t>62,4 %</t>
+  </si>
+  <si>
+    <t>33,6 %</t>
+  </si>
+  <si>
+    <t>2,54 %</t>
+  </si>
+  <si>
+    <t>50,1 %</t>
+  </si>
+  <si>
+    <t>34,5 %</t>
+  </si>
+  <si>
+    <t>4,05 %</t>
+  </si>
+  <si>
+    <t>33,5 %</t>
+  </si>
+  <si>
+    <t>8,29 %</t>
+  </si>
+  <si>
+    <t>18,9 %</t>
+  </si>
+  <si>
+    <t>4,37 %</t>
+  </si>
+  <si>
+    <t>2,45 %</t>
+  </si>
+  <si>
+    <t>87,2 %</t>
+  </si>
+  <si>
+    <t>0,16 %</t>
+  </si>
+  <si>
+    <t>0 %</t>
+  </si>
+  <si>
+    <t>95,7 %</t>
+  </si>
+  <si>
+    <t>212h</t>
+  </si>
+  <si>
+    <t>284h</t>
+  </si>
+  <si>
+    <t>72,8 %</t>
+  </si>
+  <si>
+    <t>23,0 %</t>
+  </si>
+  <si>
+    <t>1,96 %</t>
+  </si>
+  <si>
+    <t>35,1 %</t>
+  </si>
+  <si>
+    <t>57,0 %</t>
+  </si>
+  <si>
+    <t>3,56 %</t>
+  </si>
+  <si>
+    <t>34,7 %</t>
+  </si>
+  <si>
+    <t>44,2 %</t>
+  </si>
+  <si>
+    <t>6,54 %</t>
+  </si>
+  <si>
+    <t>65,1 %</t>
+  </si>
+  <si>
+    <t>8,72 %</t>
+  </si>
+  <si>
+    <t>0,57 %</t>
+  </si>
+  <si>
+    <t>2,29 %</t>
+  </si>
+  <si>
+    <t>90,9 %</t>
+  </si>
+  <si>
+    <t>98,9 %</t>
+  </si>
+  <si>
+    <t>54,2 %</t>
+  </si>
+  <si>
+    <t>42,1 %</t>
+  </si>
+  <si>
+    <t>52,5 %</t>
+  </si>
+  <si>
+    <t>39,6 %</t>
+  </si>
+  <si>
+    <t>3,84 %</t>
+  </si>
+  <si>
+    <t>40,2 %</t>
+  </si>
+  <si>
+    <t>17,7 %</t>
+  </si>
+  <si>
+    <t>47,3 %</t>
+  </si>
+  <si>
+    <t>34,1 %</t>
+  </si>
+  <si>
+    <t>5,90 %</t>
+  </si>
+  <si>
+    <t>356h</t>
   </si>
 </sst>
 </file>
@@ -520,147 +631,147 @@
         <v>4</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>5</v>
+        <v>16</v>
       </c>
       <c r="B2" t="s">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="C2" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="D2" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="E2" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="F2">
-        <v>56946</v>
+        <v>77758</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D3" t="s">
         <v>21</v>
       </c>
-      <c r="C3" t="s">
+      <c r="E3" t="s">
         <v>22</v>
       </c>
-      <c r="D3" t="s">
-        <v>16</v>
-      </c>
-      <c r="E3" t="s">
-        <v>23</v>
-      </c>
       <c r="F3">
-        <v>56947</v>
+        <v>96583</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" t="s">
         <v>21</v>
       </c>
-      <c r="C4" t="s">
-        <v>22</v>
-      </c>
       <c r="D4" t="s">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="E4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F4">
-        <v>56948</v>
+        <v>53891</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B5" t="s">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="C5" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D5" t="s">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="E5" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="F5">
-        <v>56949</v>
+        <v>67110</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B6" t="s">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="C6" t="s">
-        <v>12</v>
+        <v>28</v>
       </c>
       <c r="D6" t="s">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="E6" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="F6">
-        <v>81646</v>
+        <v>42827</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B7" t="s">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="C7" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
       <c r="D7" t="s">
-        <v>24</v>
+        <v>31</v>
       </c>
       <c r="E7" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="F7">
-        <v>81647</v>
+        <v>59701</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="B8" t="s">
-        <v>21</v>
+        <v>32</v>
       </c>
       <c r="C8" t="s">
-        <v>12</v>
+        <v>33</v>
       </c>
       <c r="D8" t="s">
-        <v>24</v>
+        <v>34</v>
       </c>
       <c r="E8" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="F8">
-        <v>81648</v>
+        <v>182143</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
@@ -668,19 +779,19 @@
         <v>5</v>
       </c>
       <c r="B9" t="s">
-        <v>19</v>
+        <v>32</v>
       </c>
       <c r="C9" t="s">
-        <v>26</v>
+        <v>36</v>
       </c>
       <c r="D9" t="s">
-        <v>27</v>
+        <v>37</v>
       </c>
       <c r="E9" t="s">
-        <v>18</v>
+        <v>38</v>
       </c>
       <c r="F9">
-        <v>21831</v>
+        <v>148860</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
@@ -688,19 +799,19 @@
         <v>6</v>
       </c>
       <c r="B10" t="s">
-        <v>19</v>
+        <v>32</v>
       </c>
       <c r="C10" t="s">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="D10" t="s">
-        <v>29</v>
+        <v>40</v>
       </c>
       <c r="E10" t="s">
-        <v>30</v>
+        <v>41</v>
       </c>
       <c r="F10">
-        <v>49180</v>
+        <v>59078</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
@@ -708,19 +819,19 @@
         <v>7</v>
       </c>
       <c r="B11" t="s">
-        <v>19</v>
+        <v>32</v>
       </c>
       <c r="C11" t="s">
-        <v>31</v>
+        <v>42</v>
       </c>
       <c r="D11" t="s">
-        <v>32</v>
+        <v>43</v>
       </c>
       <c r="E11" t="s">
-        <v>33</v>
+        <v>44</v>
       </c>
       <c r="F11">
-        <v>35592</v>
+        <v>36952</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
@@ -728,19 +839,19 @@
         <v>8</v>
       </c>
       <c r="B12" t="s">
-        <v>19</v>
+        <v>32</v>
       </c>
       <c r="C12" t="s">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="D12" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="E12" t="s">
-        <v>36</v>
+        <v>47</v>
       </c>
       <c r="F12">
-        <v>16233</v>
+        <v>7408</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
@@ -748,239 +859,239 @@
         <v>9</v>
       </c>
       <c r="B13" t="s">
-        <v>19</v>
+        <v>32</v>
       </c>
       <c r="C13" t="s">
-        <v>37</v>
+        <v>48</v>
       </c>
       <c r="D13" t="s">
-        <v>15</v>
+        <v>49</v>
       </c>
       <c r="E13" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="F13">
-        <v>64769</v>
+        <v>24709</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="B14" t="s">
-        <v>19</v>
+        <v>67</v>
       </c>
       <c r="C14" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D14" t="s">
-        <v>40</v>
+        <v>51</v>
       </c>
       <c r="E14" t="s">
-        <v>41</v>
+        <v>52</v>
       </c>
       <c r="F14">
-        <v>46885</v>
+        <v>42415</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="B15" t="s">
-        <v>19</v>
+        <v>67</v>
       </c>
       <c r="C15" t="s">
-        <v>42</v>
+        <v>53</v>
       </c>
       <c r="D15" t="s">
-        <v>43</v>
+        <v>54</v>
       </c>
       <c r="E15" t="s">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="F15">
-        <v>43695</v>
+        <v>39216</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B16" t="s">
-        <v>45</v>
+        <v>67</v>
       </c>
       <c r="C16" t="s">
-        <v>46</v>
+        <v>14</v>
       </c>
       <c r="D16" t="s">
-        <v>47</v>
+        <v>56</v>
       </c>
       <c r="E16" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="F16">
-        <v>180773</v>
+        <v>68223</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B17" t="s">
-        <v>45</v>
+        <v>67</v>
       </c>
       <c r="C17" t="s">
-        <v>49</v>
+        <v>58</v>
       </c>
       <c r="D17" t="s">
-        <v>50</v>
+        <v>59</v>
       </c>
       <c r="E17" t="s">
-        <v>51</v>
+        <v>60</v>
       </c>
       <c r="F17">
-        <v>129156</v>
+        <v>134012</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B18" t="s">
-        <v>45</v>
+        <v>67</v>
       </c>
       <c r="C18" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="D18" t="s">
-        <v>53</v>
+        <v>62</v>
       </c>
       <c r="E18" t="s">
-        <v>54</v>
+        <v>63</v>
       </c>
       <c r="F18">
-        <v>148703</v>
+        <v>1476</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B19" t="s">
-        <v>45</v>
+        <v>67</v>
       </c>
       <c r="C19" t="s">
-        <v>55</v>
+        <v>64</v>
       </c>
       <c r="D19" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="E19" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="F19">
-        <v>241764</v>
+        <v>3389</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="B20" t="s">
-        <v>45</v>
+        <v>86</v>
       </c>
       <c r="C20" t="s">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="D20" t="s">
-        <v>59</v>
+        <v>69</v>
       </c>
       <c r="E20" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="F20">
-        <v>161140</v>
+        <v>138881</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="B21" t="s">
-        <v>45</v>
+        <v>86</v>
       </c>
       <c r="C21" t="s">
-        <v>61</v>
+        <v>71</v>
       </c>
       <c r="D21" t="s">
-        <v>62</v>
+        <v>72</v>
       </c>
       <c r="E21" t="s">
-        <v>14</v>
+        <v>73</v>
       </c>
       <c r="F21">
-        <v>94458</v>
+        <v>77772</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="B22" t="s">
-        <v>45</v>
+        <v>86</v>
       </c>
       <c r="C22" t="s">
-        <v>63</v>
+        <v>74</v>
       </c>
       <c r="D22" t="s">
-        <v>64</v>
+        <v>75</v>
       </c>
       <c r="E22" t="s">
-        <v>65</v>
+        <v>76</v>
       </c>
       <c r="F22">
-        <v>16774</v>
+        <v>22189</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B23" t="s">
-        <v>20</v>
+        <v>86</v>
       </c>
       <c r="C23" t="s">
-        <v>17</v>
+        <v>77</v>
       </c>
       <c r="D23" t="s">
-        <v>66</v>
+        <v>78</v>
       </c>
       <c r="E23" t="s">
-        <v>67</v>
+        <v>79</v>
       </c>
       <c r="F23">
-        <v>64070</v>
+        <v>15860</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B24" t="s">
-        <v>20</v>
+        <v>86</v>
       </c>
       <c r="C24" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="D24" t="s">
-        <v>69</v>
+        <v>81</v>
       </c>
       <c r="E24" t="s">
-        <v>70</v>
+        <v>82</v>
       </c>
       <c r="F24">
-        <v>36164</v>
+        <v>584</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.2">
@@ -988,132 +1099,261 @@
         <v>9</v>
       </c>
       <c r="B25" t="s">
-        <v>20</v>
+        <v>86</v>
       </c>
       <c r="C25" t="s">
-        <v>71</v>
+        <v>83</v>
       </c>
       <c r="D25" t="s">
-        <v>72</v>
+        <v>84</v>
       </c>
       <c r="E25" t="s">
-        <v>73</v>
+        <v>85</v>
       </c>
       <c r="F25">
-        <v>91388</v>
+        <v>634</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="B26" t="s">
-        <v>20</v>
+        <v>87</v>
       </c>
       <c r="C26" t="s">
-        <v>74</v>
+        <v>88</v>
       </c>
       <c r="D26" t="s">
-        <v>75</v>
+        <v>89</v>
       </c>
       <c r="E26" t="s">
-        <v>76</v>
+        <v>90</v>
       </c>
       <c r="F26">
-        <v>46770</v>
+        <v>54946</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="C27"/>
-      <c r="D27"/>
-      <c r="E27"/>
+      <c r="A27" t="s">
+        <v>5</v>
+      </c>
+      <c r="B27" t="s">
+        <v>87</v>
+      </c>
+      <c r="C27" t="s">
+        <v>91</v>
+      </c>
+      <c r="D27" t="s">
+        <v>92</v>
+      </c>
+      <c r="E27" t="s">
+        <v>93</v>
+      </c>
+      <c r="F27">
+        <v>136842</v>
+      </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="C28"/>
-      <c r="D28"/>
-      <c r="E28"/>
+      <c r="A28" t="s">
+        <v>6</v>
+      </c>
+      <c r="B28" t="s">
+        <v>87</v>
+      </c>
+      <c r="C28" t="s">
+        <v>94</v>
+      </c>
+      <c r="D28" t="s">
+        <v>95</v>
+      </c>
+      <c r="E28" t="s">
+        <v>96</v>
+      </c>
+      <c r="F28">
+        <v>7542</v>
+      </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="C29"/>
-      <c r="D29"/>
-      <c r="E29"/>
+      <c r="A29" t="s">
+        <v>7</v>
+      </c>
+      <c r="B29" t="s">
+        <v>87</v>
+      </c>
+      <c r="C29" t="s">
+        <v>97</v>
+      </c>
+      <c r="D29" t="s">
+        <v>13</v>
+      </c>
+      <c r="E29" t="s">
+        <v>98</v>
+      </c>
+      <c r="F29">
+        <v>20465</v>
+      </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="C30"/>
-      <c r="D30"/>
-      <c r="E30"/>
-      <c r="F30" s="3"/>
+      <c r="A30" t="s">
+        <v>8</v>
+      </c>
+      <c r="B30" t="s">
+        <v>87</v>
+      </c>
+      <c r="C30" t="s">
+        <v>99</v>
+      </c>
+      <c r="D30" t="s">
+        <v>100</v>
+      </c>
+      <c r="E30" t="s">
+        <v>101</v>
+      </c>
+      <c r="F30">
+        <v>354</v>
+      </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="C31"/>
-      <c r="D31"/>
-      <c r="E31"/>
-      <c r="F31" s="3"/>
+      <c r="A31" t="s">
+        <v>9</v>
+      </c>
+      <c r="B31" t="s">
+        <v>87</v>
+      </c>
+      <c r="C31" t="s">
+        <v>84</v>
+      </c>
+      <c r="D31" t="s">
+        <v>84</v>
+      </c>
+      <c r="E31" t="s">
+        <v>102</v>
+      </c>
+      <c r="F31">
+        <v>370</v>
+      </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="C32"/>
-      <c r="D32"/>
-      <c r="E32"/>
-      <c r="F32" s="3"/>
-    </row>
-    <row r="33" spans="3:6" x14ac:dyDescent="0.2">
-      <c r="C33"/>
-      <c r="D33"/>
-      <c r="E33"/>
-      <c r="F33" s="3"/>
-    </row>
-    <row r="34" spans="3:6" x14ac:dyDescent="0.2">
-      <c r="C34"/>
-      <c r="D34"/>
-      <c r="E34"/>
-      <c r="F34" s="3"/>
-    </row>
-    <row r="35" spans="3:6" x14ac:dyDescent="0.2">
-      <c r="C35"/>
-      <c r="D35"/>
-      <c r="E35"/>
-      <c r="F35" s="3"/>
-    </row>
-    <row r="36" spans="3:6" x14ac:dyDescent="0.2">
+      <c r="A32" t="s">
+        <v>16</v>
+      </c>
+      <c r="B32" t="s">
+        <v>113</v>
+      </c>
+      <c r="C32" t="s">
+        <v>103</v>
+      </c>
+      <c r="D32" t="s">
+        <v>104</v>
+      </c>
+      <c r="E32" t="s">
+        <v>70</v>
+      </c>
+      <c r="F32">
+        <v>106583</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A33" t="s">
+        <v>5</v>
+      </c>
+      <c r="B33" t="s">
+        <v>113</v>
+      </c>
+      <c r="C33" t="s">
+        <v>105</v>
+      </c>
+      <c r="D33" t="s">
+        <v>106</v>
+      </c>
+      <c r="E33" t="s">
+        <v>107</v>
+      </c>
+      <c r="F33">
+        <v>64028</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A34" t="s">
+        <v>6</v>
+      </c>
+      <c r="B34" t="s">
+        <v>113</v>
+      </c>
+      <c r="C34" t="s">
+        <v>108</v>
+      </c>
+      <c r="D34" t="s">
+        <v>109</v>
+      </c>
+      <c r="E34" t="s">
+        <v>26</v>
+      </c>
+      <c r="F34">
+        <v>2222</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A35" t="s">
+        <v>7</v>
+      </c>
+      <c r="B35" t="s">
+        <v>113</v>
+      </c>
+      <c r="C35" t="s">
+        <v>110</v>
+      </c>
+      <c r="D35" t="s">
+        <v>111</v>
+      </c>
+      <c r="E35" t="s">
+        <v>112</v>
+      </c>
+      <c r="F35">
+        <v>148731</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
       <c r="C36"/>
       <c r="D36"/>
       <c r="E36"/>
       <c r="F36" s="3"/>
     </row>
-    <row r="37" spans="3:6" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
       <c r="F37" s="4"/>
     </row>
-    <row r="38" spans="3:6" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
       <c r="F38" s="4"/>
     </row>
-    <row r="39" spans="3:6" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
       <c r="F39" s="4"/>
     </row>
-    <row r="40" spans="3:6" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.2">
       <c r="F40" s="4"/>
     </row>
-    <row r="41" spans="3:6" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
       <c r="F41" s="4"/>
     </row>
-    <row r="42" spans="3:6" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.2">
       <c r="F42" s="4"/>
     </row>
-    <row r="43" spans="3:6" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.2">
       <c r="F43" s="4"/>
     </row>
-    <row r="44" spans="3:6" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.2">
       <c r="F44" s="4"/>
     </row>
-    <row r="45" spans="3:6" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.2">
       <c r="F45" s="4"/>
     </row>
-    <row r="46" spans="3:6" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.2">
       <c r="F46" s="1"/>
     </row>
-    <row r="47" spans="3:6" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.2">
       <c r="F47" s="1"/>
     </row>
-    <row r="48" spans="3:6" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.2">
       <c r="F48" s="1"/>
     </row>
     <row r="49" spans="6:6" x14ac:dyDescent="0.2">

</xml_diff>